<commit_message>
Write the Excel files identically on every machine
openpyxl formats its XML with lxml when lxml happens to be installed and with Python's own
library otherwise, so the same data gave different bytes on different machines. The package
now always selects Python's own library before openpyxl is imported. The Excel check also
tolerates LibreOffice holding its temporary files open, which happens on Windows.
</commit_message>
<xml_diff>
--- a/data/sample/marketing_spend.xlsx
+++ b/data/sample/marketing_spend.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spend 2024-26" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Spend 2024-26" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>